<commit_message>
Updated to fetch jira data via api
</commit_message>
<xml_diff>
--- a/Data/IssuesSourceFiles/Jira-issues.csv.xlsx
+++ b/Data/IssuesSourceFiles/Jira-issues.csv.xlsx
@@ -22186,7 +22186,7 @@
         <v>46115.643750000003</v>
       </c>
     </row>
-    <row r="31" spans="1:432" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:432" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>625</v>
       </c>
@@ -22299,7 +22299,7 @@
         <v>46114.506944444445</v>
       </c>
     </row>
-    <row r="32" spans="1:432" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:432" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>634</v>
       </c>
@@ -23034,7 +23034,7 @@
         <v>46112.896527777775</v>
       </c>
     </row>
-    <row r="35" spans="1:432" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:432" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>764</v>
       </c>
@@ -23171,7 +23171,7 @@
         <v>46112.850694444445</v>
       </c>
     </row>
-    <row r="36" spans="1:432" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:432" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>215</v>
       </c>
@@ -23323,7 +23323,7 @@
         <v>46112.647222222222</v>
       </c>
     </row>
-    <row r="37" spans="1:432" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:432" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>786</v>
       </c>
@@ -23463,7 +23463,7 @@
         <v>46112.649305555555</v>
       </c>
     </row>
-    <row r="38" spans="1:432" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:432" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>800</v>
       </c>
@@ -24553,7 +24553,7 @@
         <v>46118.421527777777</v>
       </c>
     </row>
-    <row r="46" spans="1:432" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:432" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>889</v>
       </c>

</xml_diff>